<commit_message>
Solved few more questions
</commit_message>
<xml_diff>
--- a/Leetcode solutions list.xlsx
+++ b/Leetcode solutions list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rushikesh\leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4AA1FCE-4686-4F02-8AA0-7B111C71A2DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47231276-BC57-46D6-8647-C518EA75743F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="4" xr2:uid="{E386DD19-1778-44D0-BE04-CA79BC411B80}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{E386DD19-1778-44D0-BE04-CA79BC411B80}"/>
   </bookViews>
   <sheets>
     <sheet name="Arrays &amp; hashing" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Binary Search" sheetId="7" r:id="rId5"/>
     <sheet name="Linked List" sheetId="4" r:id="rId6"/>
     <sheet name="Trees" sheetId="5" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="207">
   <si>
     <t>Problem</t>
   </si>
@@ -611,9 +612,6 @@
 then for size number of iterations we will get the element and put the value to the array list and add the arraylist tot he final result. now add the root.left and root.right if they are not null</t>
   </si>
   <si>
-    <t>https://leetcode.com/problems/binary-tree-right-side-view/</t>
-  </si>
-  <si>
     <t>Logic will be same as Binary tree level order treversal
 solution one :- update the value at level-1 index in the list with the node.vale
 solution 2:- instead of adding all the ements to the list we will just add last element to the list which is the right side</t>
@@ -814,6 +812,110 @@
   </si>
   <si>
     <t>leetcode/src/hard/MedianOfTwoSortedArrays.java at main · reaper131299/leetcode</t>
+  </si>
+  <si>
+    <t>Binary Tree Right Side View - LeetCode</t>
+  </si>
+  <si>
+    <t>Count Good Nodes in Binary Tree - LeetCode</t>
+  </si>
+  <si>
+    <t>Use recursion
+Keep tack of prev max.
+if current value is greated than or equal to prev max increment the counter and prev max</t>
+  </si>
+  <si>
+    <t>leetcode/src/leetcode/medium/CountGoodNodesInBinaryTree.java at main · reaper131299/leetcode</t>
+  </si>
+  <si>
+    <t>Validate Binary Search Tree - LeetCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use recursion
+we will use left and right boundary to check if node is valid or not.
+Left node should be between left boundary and parent root node. Same with with right boundary </t>
+  </si>
+  <si>
+    <t>Initialize with long as the constrains say the vlaues may be 
+interger.Min_value and integer.maxvalue.</t>
+  </si>
+  <si>
+    <t>leetcode/src/leetcode/medium/ValidateBinarySearchTree.java at main · reaper131299/leetcode</t>
+  </si>
+  <si>
+    <t>Kth Smallest Element in a BST - LeetCode</t>
+  </si>
+  <si>
+    <t>We can create in order traversal to create the array and get k-1 th element.
+2nd faster solution:-
+we can have stack. We will do in order traversal iteratively so that we don’t have to go through entire binary tree.
+Keep track of current node.
+Keep on adding root to the stack until it becomes null and move the root to root.left
+if root == null that means we have reached the end of the left sub ree.
+node = pop the top element from stack. increment the counter check if the counter == k if yes return the value.
+else root == root.right</t>
+  </si>
+  <si>
+    <t>leetcode/src/leetcode/medium/KthSmallestElementInABST.java at main · reaper131299/leetcode</t>
+  </si>
+  <si>
+    <t>Construct Binary Tree from Preorder and Inorder Traversal - LeetCode</t>
+  </si>
+  <si>
+    <t>Use recursion. 
+we can iterate over the preorder array using a global counter n. And increment the counter as we recursively call the method.
+We can use left and and right pointer. 
+If left pointer is &gt;right poiner the element is null. 
+We will get the value preorder[n] and create a node.
+we will the increment the pointer.
+we will then find the index of same value in inorder array.
+then node.left = left pointer, index-1
+node.right = index+1, right pointer
+return node</t>
+  </si>
+  <si>
+    <t>leetcode/src/leetcode/medium/ConstructBinaryTreeFromPreorderAndInorderTraversal.java at main · reaper131299/leetcode</t>
+  </si>
+  <si>
+    <t>Binary Tree Maximum Path Sum - LeetCode</t>
+  </si>
+  <si>
+    <t>use recursion.
+To find amx path you have to find leftMaxPath and rightMaxPath. We will do that recursively.
+Once we get right and left max path. We will do 3 comparisons.
+Max1 = Math.max(root+leftMaxPath, root+rightMaxPath)
+Max2 = Math.max(max1, root+leftMaxPath+rightMaxPath)
+Max3 = Math.max(max2, root)
+this is because any path in the entire binary tree could be max(even the root itself max3).
+Now tack the res with max3.
+return Max between root+leftMaxPath, root+rightMaxPath and root.</t>
+  </si>
+  <si>
+    <t>even the node itself can be the max path.</t>
+  </si>
+  <si>
+    <t>leetcode/src/leetcode/hard/BinaryTreeMaximumPathSum.java at main · reaper131299/leetcode</t>
+  </si>
+  <si>
+    <t>Serialize and Deserialize Binary Tree - LeetCode</t>
+  </si>
+  <si>
+    <t>use iterations
+Serialization :- we can use linked list as queue.
+String builder to generate the string.
+Add elements to the queue. Get the size of queue. And for size iterations poll the first element of queue and add the left and right elements to queue. add the polled element to the string builder with delimeter.
+deserialize:-
+split the strign based on the delimeter.
+take the first element create node, initialize left and right pointer as 1,2.
+Add the first element to queue.
+get the element at left and right index from string[] create a node if string != null. and let to left and right respectively add the elemnts to queue, increment the left and right pointer by 2. if string == null then do not add it to queue.</t>
+  </si>
+  <si>
+    <t>while serializing check if polled element is null or not.
+While deserializing check for left and right ements and then increment the left and right counter by 2 only once</t>
+  </si>
+  <si>
+    <t>leetcode/src/leetcode/hard/SerializeAndDeserializeBinaryTree.java at main · reaper131299/leetcode</t>
   </si>
 </sst>
 </file>
@@ -887,7 +989,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -899,9 +1001,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1754,121 +1853,121 @@
     </row>
     <row r="2" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="D4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>158</v>
-      </c>
       <c r="D7" t="s">
         <v>6</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="D8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -1923,121 +2022,121 @@
     </row>
     <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
         <v>165</v>
       </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="D4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>176</v>
-      </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" t="s">
         <v>178</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="1" t="s">
         <v>184</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2307,7 +2406,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{221076E7-411D-4D35-96C4-18B4D9A10664}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -2472,19 +2571,121 @@
     </row>
     <row r="10" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>137</v>
+        <v>185</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D10" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D10" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>139</v>
+    </row>
+    <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="144" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D13" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D15" t="s">
+        <v>201</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -2506,7 +2707,29 @@
     <hyperlink ref="A9" r:id="rId15" display="https://leetcode.com/problems/binary-tree-level-order-traversal/description/" xr:uid="{9F3DEB1D-237C-40EA-8C8A-953A8E9EECBB}"/>
     <hyperlink ref="E9" r:id="rId16" display="https://github.com/reaper131299/leetcode/blob/main/src/medium/BinaryTreeLevelOrderTraversal.java" xr:uid="{487753B9-120D-430E-928C-4AC6C93B9594}"/>
     <hyperlink ref="E10" r:id="rId17" display="https://github.com/reaper131299/leetcode/blob/main/src/medium/BinaryTreeRightSideView.java" xr:uid="{53831DB9-BF96-42A5-B864-65395160A8A9}"/>
+    <hyperlink ref="A10" r:id="rId18" display="https://leetcode.com/problems/binary-tree-right-side-view/" xr:uid="{115D2F38-1252-4D16-B0C2-93CCA67DE81D}"/>
+    <hyperlink ref="A11" r:id="rId19" display="https://leetcode.com/problems/count-good-nodes-in-binary-tree/description/" xr:uid="{18110539-52DF-4826-818F-28F90B19322E}"/>
+    <hyperlink ref="E11" r:id="rId20" display="https://github.com/reaper131299/leetcode/blob/main/src/leetcode/medium/CountGoodNodesInBinaryTree.java" xr:uid="{2788A78D-57DB-4DB4-8174-42D16F3EA2D4}"/>
+    <hyperlink ref="A12" r:id="rId21" display="https://leetcode.com/problems/validate-binary-search-tree/description/" xr:uid="{46AE653D-3EA1-433C-B83E-B0DE59DE7B35}"/>
+    <hyperlink ref="E12" r:id="rId22" display="https://github.com/reaper131299/leetcode/blob/main/src/leetcode/medium/ValidateBinarySearchTree.java" xr:uid="{ABC0CBFA-258C-46C6-A0AB-0FAE7A013F53}"/>
+    <hyperlink ref="A13" r:id="rId23" display="https://leetcode.com/problems/kth-smallest-element-in-a-bst/" xr:uid="{2F6C522C-A52F-4F50-813F-B6BF74A3E03A}"/>
+    <hyperlink ref="E13" r:id="rId24" display="https://github.com/reaper131299/leetcode/blob/main/src/leetcode/medium/KthSmallestElementInABST.java" xr:uid="{9AA303EF-7784-4B51-87CF-09435E24FBE2}"/>
+    <hyperlink ref="A14" r:id="rId25" display="https://leetcode.com/problems/construct-binary-tree-from-preorder-and-inorder-traversal/description/" xr:uid="{284C98AC-B250-4C49-8872-1D53FDD13B2B}"/>
+    <hyperlink ref="E14" r:id="rId26" display="https://github.com/reaper131299/leetcode/blob/main/src/leetcode/medium/ConstructBinaryTreeFromPreorderAndInorderTraversal.java" xr:uid="{764BE3F3-2C30-45A6-9ECA-6626BA876DDD}"/>
+    <hyperlink ref="A15" r:id="rId27" display="https://leetcode.com/problems/binary-tree-maximum-path-sum/" xr:uid="{25D2E43C-7E6E-494E-9DAF-B3B637F3B4E6}"/>
+    <hyperlink ref="E15" r:id="rId28" display="https://github.com/reaper131299/leetcode/blob/main/src/leetcode/hard/BinaryTreeMaximumPathSum.java" xr:uid="{5A0E4BAB-0370-4507-99CA-7C324B39E92D}"/>
+    <hyperlink ref="A16" r:id="rId29" display="https://leetcode.com/problems/serialize-and-deserialize-binary-tree/" xr:uid="{CD29A3CB-8DF8-4327-81F7-464C65A86E24}"/>
+    <hyperlink ref="E16" r:id="rId30" display="https://github.com/reaper131299/leetcode/blob/main/src/leetcode/hard/SerializeAndDeserializeBinaryTree.java" xr:uid="{88FDAA8C-64A9-4638-9948-9CED05F90F4C}"/>
   </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDEC9266-3BF5-42C1-9773-E32B48ADAE3F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>